<commit_message>
Add MCC 32-point (option B) quote and internal margin files; align decks and comparison sheet to option B
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjFrCobQqqs1TtLcuKd8BA
</commit_message>
<xml_diff>
--- a/MCC_32점_비교.xlsx
+++ b/MCC_32점_비교.xlsx
@@ -3650,7 +3650,7 @@
         <v>43</v>
       </c>
       <c r="D27" s="29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E27" s="17" t="n">
         <v>32</v>
@@ -3802,7 +3802,7 @@
         <v>28</v>
       </c>
       <c r="D31" s="29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31" s="17" t="n">
         <v>16</v>
@@ -3823,11 +3823,11 @@
       </c>
       <c r="L31" s="22" t="n">
         <f aca="false">D31*K31</f>
-        <v>0</v>
+        <v>79800</v>
       </c>
       <c r="M31" s="31" t="str">
-        <f aca="false">IF(AND(D31&gt;0,H31="",J31=""),"▶ 단가 입력 필요","필요 시 수량 입력")</f>
-        <v>필요 시 수량 입력</v>
+        <f aca="false">IF(AND(D31&gt;0,H31="",J31=""),"▶ 단가 입력 필요","")</f>
+        <v/>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="D35" s="32" t="n">
         <f aca="false">2*(D27+D28)</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E35" s="17"/>
       <c r="F35" s="17"/>
@@ -4021,7 +4021,7 @@
       <c r="D37" s="25"/>
       <c r="E37" s="26" t="n">
         <f aca="false">SUMPRODUCT($D$26:$D$36,E26:E36)</f>
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="F37" s="26" t="n">
         <f aca="false">SUMPRODUCT($D$26:$D$36,F26:F36)</f>
@@ -4037,7 +4037,7 @@
       <c r="K37" s="25"/>
       <c r="L37" s="27" t="n">
         <f aca="false">SUM(L26:L36)</f>
-        <v>549650</v>
+        <v>629450</v>
       </c>
       <c r="M37" s="25"/>
     </row>
@@ -4106,7 +4106,7 @@
       <c r="C42" s="6"/>
       <c r="D42" s="37" t="n">
         <f aca="false">E37</f>
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="E42" s="13" t="s">
         <v>58</v>
@@ -4316,7 +4316,7 @@
       <c r="C51" s="41"/>
       <c r="D51" s="21" t="n">
         <f aca="false">$L$37</f>
-        <v>549650</v>
+        <v>629450</v>
       </c>
       <c r="E51" s="21"/>
       <c r="F51" s="21" t="n">
@@ -4326,16 +4326,16 @@
       <c r="G51" s="21"/>
       <c r="H51" s="22" t="n">
         <f aca="false">F51-D51</f>
-        <v>900350</v>
+        <v>820550</v>
       </c>
       <c r="I51" s="22"/>
       <c r="J51" s="38" t="n">
         <f aca="false">IF(F51=0,"",H51/F51)</f>
-        <v>0.620931034482759</v>
+        <v>0.565896551724138</v>
       </c>
       <c r="K51" s="21" t="n">
         <f aca="false">H51*$D$8</f>
-        <v>90035000</v>
+        <v>82055000</v>
       </c>
       <c r="L51" s="39" t="n">
         <f aca="false">IF($D$6=0,"",F51/$D$6-1)</f>
@@ -4353,7 +4353,7 @@
       <c r="C52" s="41"/>
       <c r="D52" s="21" t="n">
         <f aca="false">$L$37</f>
-        <v>549650</v>
+        <v>629450</v>
       </c>
       <c r="E52" s="21"/>
       <c r="F52" s="21" t="n">
@@ -4363,16 +4363,16 @@
       <c r="G52" s="21"/>
       <c r="H52" s="22" t="n">
         <f aca="false">F52-D52</f>
-        <v>900350</v>
+        <v>820550</v>
       </c>
       <c r="I52" s="22"/>
       <c r="J52" s="38" t="n">
         <f aca="false">IF(F52=0,"",H52/F52)</f>
-        <v>0.620931034482759</v>
+        <v>0.565896551724138</v>
       </c>
       <c r="K52" s="21" t="n">
         <f aca="false">H52*$D$8</f>
-        <v>90035000</v>
+        <v>82055000</v>
       </c>
       <c r="L52" s="39" t="n">
         <f aca="false">IF($D$6=0,"",F52/$D$6-1)</f>
@@ -4390,7 +4390,7 @@
       <c r="C53" s="41"/>
       <c r="D53" s="21" t="n">
         <f aca="false">$L$37</f>
-        <v>549650</v>
+        <v>629450</v>
       </c>
       <c r="E53" s="21"/>
       <c r="F53" s="21" t="n">
@@ -4400,16 +4400,16 @@
       <c r="G53" s="21"/>
       <c r="H53" s="22" t="n">
         <f aca="false">F53-D53</f>
-        <v>620350</v>
+        <v>540550</v>
       </c>
       <c r="I53" s="22"/>
       <c r="J53" s="38" t="n">
         <f aca="false">IF(F53=0,"",H53/F53)</f>
-        <v>0.530213675213675</v>
+        <v>0.462008547008547</v>
       </c>
       <c r="K53" s="21" t="n">
         <f aca="false">H53*$D$8</f>
-        <v>62035000</v>
+        <v>54055000</v>
       </c>
       <c r="L53" s="39" t="n">
         <f aca="false">IF($D$6=0,"",F53/$D$6-1)</f>
@@ -4427,7 +4427,7 @@
       <c r="C55" s="6"/>
       <c r="D55" s="27" t="n">
         <f aca="false">$L$22-$L$37</f>
-        <v>677250</v>
+        <v>597450</v>
       </c>
       <c r="E55" s="27"/>
       <c r="F55" s="27"/>
@@ -4449,7 +4449,7 @@
       <c r="C56" s="6"/>
       <c r="D56" s="27" t="n">
         <f aca="false">D55*$D$8</f>
-        <v>67725000</v>
+        <v>59745000</v>
       </c>
       <c r="E56" s="27"/>
       <c r="F56" s="27"/>
@@ -4469,7 +4469,7 @@
       <c r="C57" s="6"/>
       <c r="D57" s="27" t="n">
         <f aca="false">ROUNDUP($L$37/(1-$D$11),-3)</f>
-        <v>647000</v>
+        <v>741000</v>
       </c>
       <c r="E57" s="27"/>
       <c r="F57" s="27"/>
@@ -4513,7 +4513,7 @@
       <c r="C59" s="6"/>
       <c r="D59" s="27" t="n">
         <f aca="false">$L$37-D58</f>
-        <v>-444850</v>
+        <v>-365050</v>
       </c>
       <c r="E59" s="27"/>
       <c r="F59" s="27"/>

</xml_diff>